<commit_message>
Add refund/loan columns to monthly breakdown and duplicate detection
- Add refund_deposits and loan_credit_deposits fields to MonthlyBreakdown model
- Update Gemini prompt with explicit per-category sums and deduplication logic
- Add "Remboursements" and "Prêts/crédit" columns to Detail mensuel sheet
- Regenerate Excel template to match new column layout
- Update test fixtures with new fields

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/mortgage_mcp/templates/grille_revenu_autonome.xlsx
+++ b/src/mortgage_mcp/templates/grille_revenu_autonome.xlsx
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -567,10 +567,12 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -601,20 +603,30 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>Remboursements</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Prêts/crédit</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
           <t>Autres</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Retraits</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Revenu net</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Nb dépôts</t>
         </is>

</xml_diff>

<commit_message>
Add account column to Depots sheet for multi-account traceability
- Add account field to Deposit and Withdrawal models
- Instruct Gemini to tag each transaction with "Institution XX99" format
- Add "Compte" column to Depots sheet (between Date and Description)
- Update template to match new column layout

Helps mortgage brokers validate transactions across multiple accounts.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/mortgage_mcp/templates/grille_revenu_autonome.xlsx
+++ b/src/mortgage_mcp/templates/grille_revenu_autonome.xlsx
@@ -643,13 +643,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -660,15 +661,20 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
+          <t>Compte</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Montant</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Catégorie</t>
         </is>

</xml_diff>